<commit_message>
Fix UG marking rate to exact 1/3h (20 min/script) and regenerate baseline
Update marking_hours_per_script.manual.ug in workload_parameters.yaml from
0.33 to 1/3 for full precision, matching the corrected rate in
Work Allocation Model.docx (Table 4: "1/3 (20 min)"). Regenerate baseline
outputs to reflect the corrected marking hours across all staff reports.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/baseline/Staff workload model.xlsx
+++ b/baseline/Staff workload model.xlsx
@@ -913,10 +913,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1014.1</v>
+        <v>1014.3</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>344.8</v>
+        <v>345</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>412.2</v>
@@ -960,10 +960,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>1291.256</v>
+        <v>1291.3</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>343.656</v>
+        <v>343.7</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>444.2</v>
@@ -1007,10 +1007,10 @@
         <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>811.76</v>
+        <v>812.2666666666667</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>204.36</v>
+        <v>204.8666666666667</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>268.2</v>
@@ -1054,10 +1054,10 @@
         <v>1</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>872.8866666666667</v>
+        <v>873.6333333333333</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>451.5866666666667</v>
+        <v>452.3333333333333</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>164.2</v>
@@ -1101,10 +1101,10 @@
         <v>1</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1061.264</v>
+        <v>1061.466666666667</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>241.664</v>
+        <v>241.8666666666666</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>644.6000000000001</v>
@@ -1148,10 +1148,10 @@
         <v>1</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1023.549333333333</v>
+        <v>1023.633333333333</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>416.1493333333333</v>
+        <v>416.2333333333333</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>268.2</v>
@@ -1195,10 +1195,10 @@
         <v>1</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>1155.914</v>
+        <v>1156.65</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>529.364</v>
+        <v>530.1</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>164.2</v>
@@ -1242,10 +1242,10 @@
         <v>1</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>659.9159999999999</v>
+        <v>660</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>238.616</v>
+        <v>238.7</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>164.2</v>
@@ -1289,10 +1289,10 @@
         <v>1</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>663.6613333333333</v>
+        <v>664.0666666666666</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>212.4613333333333</v>
+        <v>212.8666666666667</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>276.2</v>
@@ -1336,10 +1336,10 @@
         <v>1</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>978.5599999999999</v>
+        <v>978.76</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>223.8</v>
+        <v>224</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>579.76</v>
@@ -1383,10 +1383,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>749.6666666666667</v>
+        <v>750.0333333333333</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>410.4666666666667</v>
+        <v>410.8333333333333</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>164.2</v>
@@ -1430,10 +1430,10 @@
         <v>1</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>775.8266666666666</v>
+        <v>776.7</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>436.6266666666667</v>
+        <v>437.5</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>164.2</v>
@@ -1477,10 +1477,10 @@
         <v>1</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>1112.058666666667</v>
+        <v>1112.9</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>348.4586666666667</v>
+        <v>349.3</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>260.2</v>
@@ -1524,10 +1524,10 @@
         <v>1</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1256.2</v>
+        <v>1256.4</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>296.8</v>
+        <v>297</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>620.2</v>
@@ -1571,10 +1571,10 @@
         <v>1</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>1340.030666666667</v>
+        <v>1340.1</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>50.13066666666666</v>
+        <v>50.2</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>1114.9</v>
@@ -1618,10 +1618,10 @@
         <v>1</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>712.1453333333334</v>
+        <v>713</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>372.9453333333333</v>
+        <v>373.8</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>164.2</v>
@@ -1665,10 +1665,10 @@
         <v>1</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>458.16</v>
+        <v>458.2</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>70.96000000000001</v>
+        <v>71</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>212.2</v>
@@ -1712,10 +1712,10 @@
         <v>1</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>2133.82</v>
+        <v>2134.02</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>82.3</v>
+        <v>82.5</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>1794.42</v>
@@ -1806,10 +1806,10 @@
         <v>1</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1443.926</v>
+        <v>1444</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>99.726</v>
+        <v>99.8</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>348.2</v>
@@ -1853,10 +1853,10 @@
         <v>1</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>930.6573333333333</v>
+        <v>931.4333333333334</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>345.1573333333333</v>
+        <v>345.9333333333333</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>246.3</v>
@@ -1900,10 +1900,10 @@
         <v>1</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>972.532</v>
+        <v>972.9</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>551.232</v>
+        <v>551.6</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>164.2</v>
@@ -1947,10 +1947,10 @@
         <v>1</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>1485.261333333333</v>
+        <v>1485.666666666667</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>309.4613333333333</v>
+        <v>309.8666666666667</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>1000.8</v>
@@ -1994,10 +1994,10 @@
         <v>1</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>855.498</v>
+        <v>855.5999999999999</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>348.298</v>
+        <v>348.4</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>332.2</v>
@@ -2041,10 +2041,10 @@
         <v>1</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>985.0060000000001</v>
+        <v>985.1</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>297.606</v>
+        <v>297.7</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>348.2</v>
@@ -2135,10 +2135,10 @@
         <v>1</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>1162.505333333333</v>
+        <v>1162.933333333333</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>446.9053333333333</v>
+        <v>447.3333333333334</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>212.2</v>
@@ -2182,10 +2182,10 @@
         <v>1</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>1165.126666666667</v>
+        <v>1166</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>387.6266666666667</v>
+        <v>388.5</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>356.2</v>
@@ -2229,10 +2229,10 @@
         <v>1</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>1169.744</v>
+        <v>1170.233333333333</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>364.044</v>
+        <v>364.5333333333333</v>
       </c>
       <c r="E30" s="3" t="n">
         <v>548.6</v>
@@ -2276,10 +2276,10 @@
         <v>1</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>893.8866666666667</v>
+        <v>894.6333333333333</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>472.5866666666667</v>
+        <v>473.3333333333333</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>164.2</v>
@@ -2370,10 +2370,10 @@
         <v>1</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>1468.557333333333</v>
+        <v>1468.933333333333</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>208.5573333333333</v>
+        <v>208.9333333333333</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>428.2</v>
@@ -2417,10 +2417,10 @@
         <v>1</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>1609.757333333333</v>
+        <v>1610.133333333333</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>257.9573333333333</v>
+        <v>258.3333333333334</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>1012.6</v>
@@ -2464,10 +2464,10 @@
         <v>1</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>1288.54</v>
+        <v>1289</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>304.74</v>
+        <v>305.2</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>644.6</v>
@@ -2511,10 +2511,10 @@
         <v>1</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>1397.213333333334</v>
+        <v>1397.58</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>225.6333333333333</v>
+        <v>226</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>996.5800000000002</v>
@@ -2558,10 +2558,10 @@
         <v>1</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>1118.96</v>
+        <v>1119.4</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>479.5600000000001</v>
+        <v>480</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>300.2</v>
@@ -2648,10 +2648,10 @@
         <v>1</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>1702.497333333333</v>
+        <v>1702.933333333333</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>250.4973333333333</v>
+        <v>250.9333333333333</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>1112.8</v>
@@ -2695,10 +2695,10 @@
         <v>1</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>921.4193333333334</v>
+        <v>922.4166666666666</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>395.0693333333334</v>
+        <v>396.0666666666667</v>
       </c>
       <c r="E40" s="3" t="n">
         <v>228.2</v>
@@ -2789,10 +2789,10 @@
         <v>1</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>799.9159999999999</v>
+        <v>800</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>226.616</v>
+        <v>226.7</v>
       </c>
       <c r="E42" s="3" t="n">
         <v>398.3</v>
@@ -2836,10 +2836,10 @@
         <v>1</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>758.8133333333333</v>
+        <v>759.3666666666666</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>419.6133333333333</v>
+        <v>420.1666666666666</v>
       </c>
       <c r="E43" s="3" t="n">
         <v>164.2</v>
@@ -2883,10 +2883,10 @@
         <v>1</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>1047.239333333333</v>
+        <v>1047.383333333333</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>604.0393333333334</v>
+        <v>604.1833333333334</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>268.2</v>
@@ -2930,10 +2930,10 @@
         <v>1</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>615.9793333333333</v>
+        <v>616.4833333333333</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>276.7793333333333</v>
+        <v>277.2833333333333</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>164.2</v>
@@ -2977,10 +2977,10 @@
         <v>1</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>1193.406666666667</v>
+        <v>1193.866666666667</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>375.9066666666666</v>
+        <v>376.3666666666667</v>
       </c>
       <c r="E46" s="3" t="n">
         <v>478.3</v>
@@ -3024,10 +3024,10 @@
         <v>1</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>798.24</v>
+        <v>799.0333333333333</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>347.04</v>
+        <v>347.8333333333333</v>
       </c>
       <c r="E47" s="3" t="n">
         <v>276.2</v>
@@ -3071,10 +3071,10 @@
         <v>1</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>784.7839999999999</v>
+        <v>785</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>445.5839999999999</v>
+        <v>445.8</v>
       </c>
       <c r="E48" s="3" t="n">
         <v>164.2</v>
@@ -3118,10 +3118,10 @@
         <v>1</v>
       </c>
       <c r="C49" s="3" t="n">
-        <v>1216.17</v>
+        <v>1216.25</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>274.47</v>
+        <v>274.55</v>
       </c>
       <c r="E49" s="3" t="n">
         <v>520.4000000000001</v>
@@ -3165,10 +3165,10 @@
         <v>1</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>853.812</v>
+        <v>853.9</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>226.612</v>
+        <v>226.7</v>
       </c>
       <c r="E50" s="3" t="n">
         <v>452.2</v>
@@ -3212,10 +3212,10 @@
         <v>1</v>
       </c>
       <c r="C51" s="3" t="n">
-        <v>1183.038</v>
+        <v>1183.2</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>329.338</v>
+        <v>329.5</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>350.3</v>
@@ -3259,10 +3259,10 @@
         <v>1</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>1311.913333333333</v>
+        <v>1312.733333333333</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>608.5133333333333</v>
+        <v>609.3333333333333</v>
       </c>
       <c r="E52" s="3" t="n">
         <v>364.2</v>
@@ -3306,10 +3306,10 @@
         <v>1</v>
       </c>
       <c r="C53" s="3" t="n">
-        <v>998.854</v>
+        <v>999</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>303.454</v>
+        <v>303.6</v>
       </c>
       <c r="E53" s="3" t="n">
         <v>356.2</v>
@@ -3353,10 +3353,10 @@
         <v>1</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>1333.362</v>
+        <v>1333.55</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>359.012</v>
+        <v>359.2</v>
       </c>
       <c r="E54" s="3" t="n">
         <v>676.2</v>
@@ -3400,10 +3400,10 @@
         <v>1</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>909.908</v>
+        <v>910.5</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>408.608</v>
+        <v>409.2</v>
       </c>
       <c r="E55" s="3" t="n">
         <v>244.2</v>
@@ -3447,10 +3447,10 @@
         <v>1</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>961.78</v>
+        <v>961.8000000000001</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>148.08</v>
+        <v>148.1</v>
       </c>
       <c r="E56" s="3" t="n">
         <v>638.7</v>
@@ -3494,10 +3494,10 @@
         <v>1</v>
       </c>
       <c r="C57" s="3" t="n">
-        <v>848.994</v>
+        <v>849.1999999999999</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>411.694</v>
+        <v>411.9</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>180.2</v>
@@ -3600,7 +3600,7 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>344.8</v>
+        <v>345</v>
       </c>
       <c r="C2" s="7" t="n">
         <v>412.2</v>
@@ -3620,7 +3620,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>343.656</v>
+        <v>343.7</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>444.2</v>
@@ -3640,7 +3640,7 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>204.36</v>
+        <v>204.8666666666667</v>
       </c>
       <c r="C4" s="7" t="n">
         <v>268.2</v>
@@ -3660,7 +3660,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>451.5866666666667</v>
+        <v>452.3333333333333</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>164.2</v>
@@ -3680,7 +3680,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>241.664</v>
+        <v>241.8666666666666</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>644.6000000000001</v>
@@ -3700,7 +3700,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>416.1493333333333</v>
+        <v>416.2333333333333</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>268.2</v>
@@ -3720,7 +3720,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>529.364</v>
+        <v>530.1</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>164.2</v>
@@ -3740,7 +3740,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>238.616</v>
+        <v>238.7</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>164.2</v>
@@ -3760,7 +3760,7 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>212.4613333333333</v>
+        <v>212.8666666666667</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>276.2</v>
@@ -3780,7 +3780,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>223.8</v>
+        <v>224</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>579.76</v>
@@ -3800,7 +3800,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>410.4666666666667</v>
+        <v>410.8333333333333</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>164.2</v>
@@ -3820,7 +3820,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>436.6266666666667</v>
+        <v>437.5</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>164.2</v>
@@ -3840,7 +3840,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>348.4586666666667</v>
+        <v>349.3</v>
       </c>
       <c r="C14" s="7" t="n">
         <v>260.2</v>
@@ -3860,7 +3860,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>296.8</v>
+        <v>297</v>
       </c>
       <c r="C15" s="7" t="n">
         <v>620.2</v>
@@ -3880,7 +3880,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>50.13066666666666</v>
+        <v>50.2</v>
       </c>
       <c r="C16" s="7" t="n">
         <v>1114.9</v>
@@ -3900,7 +3900,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>372.9453333333333</v>
+        <v>373.8</v>
       </c>
       <c r="C17" s="7" t="n">
         <v>164.2</v>
@@ -3920,7 +3920,7 @@
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>70.96000000000001</v>
+        <v>71</v>
       </c>
       <c r="C18" s="7" t="n">
         <v>212.2</v>
@@ -3940,7 +3940,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>82.3</v>
+        <v>82.5</v>
       </c>
       <c r="C19" s="7" t="n">
         <v>1794.42</v>
@@ -3980,7 +3980,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>99.726</v>
+        <v>99.8</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>348.2</v>
@@ -4000,7 +4000,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>345.1573333333333</v>
+        <v>345.9333333333333</v>
       </c>
       <c r="C22" s="7" t="n">
         <v>246.3</v>
@@ -4020,7 +4020,7 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>551.232</v>
+        <v>551.6</v>
       </c>
       <c r="C23" s="7" t="n">
         <v>164.2</v>
@@ -4040,7 +4040,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>309.4613333333333</v>
+        <v>309.8666666666667</v>
       </c>
       <c r="C24" s="7" t="n">
         <v>1000.8</v>
@@ -4060,7 +4060,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>348.298</v>
+        <v>348.4</v>
       </c>
       <c r="C25" s="7" t="n">
         <v>332.2</v>
@@ -4080,7 +4080,7 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>297.606</v>
+        <v>297.7</v>
       </c>
       <c r="C26" s="7" t="n">
         <v>348.2</v>
@@ -4120,7 +4120,7 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>446.9053333333333</v>
+        <v>447.3333333333334</v>
       </c>
       <c r="C28" s="7" t="n">
         <v>212.2</v>
@@ -4140,7 +4140,7 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>387.6266666666667</v>
+        <v>388.5</v>
       </c>
       <c r="C29" s="7" t="n">
         <v>356.2</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>364.044</v>
+        <v>364.5333333333333</v>
       </c>
       <c r="C30" s="7" t="n">
         <v>548.6</v>
@@ -4180,7 +4180,7 @@
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>472.5866666666667</v>
+        <v>473.3333333333333</v>
       </c>
       <c r="C31" s="7" t="n">
         <v>164.2</v>
@@ -4220,7 +4220,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>208.5573333333333</v>
+        <v>208.9333333333333</v>
       </c>
       <c r="C33" s="7" t="n">
         <v>428.2</v>
@@ -4240,7 +4240,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>257.9573333333333</v>
+        <v>258.3333333333334</v>
       </c>
       <c r="C34" s="7" t="n">
         <v>1012.6</v>
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>304.74</v>
+        <v>305.2</v>
       </c>
       <c r="C35" s="7" t="n">
         <v>644.6</v>
@@ -4280,7 +4280,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>225.6333333333333</v>
+        <v>226</v>
       </c>
       <c r="C36" s="7" t="n">
         <v>996.5800000000002</v>
@@ -4300,7 +4300,7 @@
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>479.5600000000001</v>
+        <v>480</v>
       </c>
       <c r="C37" s="7" t="n">
         <v>300.2</v>
@@ -4340,7 +4340,7 @@
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>250.4973333333333</v>
+        <v>250.9333333333333</v>
       </c>
       <c r="C39" s="7" t="n">
         <v>1112.8</v>
@@ -4360,7 +4360,7 @@
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>395.0693333333334</v>
+        <v>396.0666666666667</v>
       </c>
       <c r="C40" s="7" t="n">
         <v>228.2</v>
@@ -4400,7 +4400,7 @@
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>226.616</v>
+        <v>226.7</v>
       </c>
       <c r="C42" s="7" t="n">
         <v>398.3</v>
@@ -4420,7 +4420,7 @@
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>419.6133333333333</v>
+        <v>420.1666666666666</v>
       </c>
       <c r="C43" s="7" t="n">
         <v>164.2</v>
@@ -4440,7 +4440,7 @@
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>604.0393333333334</v>
+        <v>604.1833333333334</v>
       </c>
       <c r="C44" s="7" t="n">
         <v>268.2</v>
@@ -4460,7 +4460,7 @@
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>276.7793333333333</v>
+        <v>277.2833333333333</v>
       </c>
       <c r="C45" s="7" t="n">
         <v>164.2</v>
@@ -4480,7 +4480,7 @@
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>375.9066666666666</v>
+        <v>376.3666666666667</v>
       </c>
       <c r="C46" s="7" t="n">
         <v>478.3</v>
@@ -4500,7 +4500,7 @@
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>347.04</v>
+        <v>347.8333333333333</v>
       </c>
       <c r="C47" s="7" t="n">
         <v>276.2</v>
@@ -4520,7 +4520,7 @@
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>445.5839999999999</v>
+        <v>445.8</v>
       </c>
       <c r="C48" s="7" t="n">
         <v>164.2</v>
@@ -4540,7 +4540,7 @@
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>274.47</v>
+        <v>274.55</v>
       </c>
       <c r="C49" s="7" t="n">
         <v>520.4000000000001</v>
@@ -4560,7 +4560,7 @@
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>226.612</v>
+        <v>226.7</v>
       </c>
       <c r="C50" s="7" t="n">
         <v>452.2</v>
@@ -4580,7 +4580,7 @@
         </is>
       </c>
       <c r="B51" s="7" t="n">
-        <v>329.338</v>
+        <v>329.5</v>
       </c>
       <c r="C51" s="7" t="n">
         <v>350.3</v>
@@ -4600,7 +4600,7 @@
         </is>
       </c>
       <c r="B52" s="7" t="n">
-        <v>608.5133333333333</v>
+        <v>609.3333333333333</v>
       </c>
       <c r="C52" s="7" t="n">
         <v>364.2</v>
@@ -4620,7 +4620,7 @@
         </is>
       </c>
       <c r="B53" s="7" t="n">
-        <v>303.454</v>
+        <v>303.6</v>
       </c>
       <c r="C53" s="7" t="n">
         <v>356.2</v>
@@ -4640,7 +4640,7 @@
         </is>
       </c>
       <c r="B54" s="7" t="n">
-        <v>359.012</v>
+        <v>359.2</v>
       </c>
       <c r="C54" s="7" t="n">
         <v>676.2</v>
@@ -4660,7 +4660,7 @@
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>408.608</v>
+        <v>409.2</v>
       </c>
       <c r="C55" s="7" t="n">
         <v>244.2</v>
@@ -4680,7 +4680,7 @@
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>148.08</v>
+        <v>148.1</v>
       </c>
       <c r="C56" s="7" t="n">
         <v>638.7</v>
@@ -4700,7 +4700,7 @@
         </is>
       </c>
       <c r="B57" s="7" t="n">
-        <v>411.694</v>
+        <v>411.9</v>
       </c>
       <c r="C57" s="7" t="n">
         <v>180.2</v>

</xml_diff>